<commit_message>
Fusionar atributos de e-Cidadania (dedup como UNA iniciativa con 2 herramientas)
Decisión del equipo: e-Cidadania cuenta como una iniciativa; la ficha del
'marcado de audiencias' consolida ahora los atributos del 'matching de ideas'
(+Participación Digital, +Referendos e Iniciativas Populares, +etapa Análisis,
+Búsqueda semántica, todos con nota de fusión). Antes el dedup descartaba esos
atributos y Brasil los perdía.

Para no contaminar la columna retrospectiva 2025 (el matching es de 2025/26),
la ficha guarda 'baseline_2025_atributos' con los valores originales del
baseline y calc_comparativo los usa al construir el set 2025.

Efecto: BR 2026 80->84 (recupera RIP como 4º tipo); 2025 intacto (75).
Prom regional 2026 = 26. Todas las planillas regeneradas.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/base_completa_ILIA2026.xlsx
+++ b/data/gates/base_completa_ILIA2026.xlsx
@@ -1407,12 +1407,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Gobernanza Colaborativa</t>
+          <t>Gobernanza Colaborativa; Participación Digital; Referendos e Iniciativas Populares</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Traducción Política</t>
+          <t>Traducción Política; Análisis</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Voz a Texto; LLM; NLP</t>
+          <t>Voz a Texto; LLM; NLP; Búsqueda semántica</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">

</xml_diff>